<commit_message>
New MkII skirts - sides still missing. Update BOM info.
</commit_message>
<xml_diff>
--- a/BOM_Trident_170_170_180.xlsx
+++ b/BOM_Trident_170_170_180.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\john\Documents\3D Printing\_Trender3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fc550a2baf076e0f/Documents/CAD Designs/3D Printers/Trender3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6325BB9C-093A-4392-B649-E98037A9BCF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="13_ncr:1_{6325BB9C-093A-4392-B649-E98037A9BCF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6AA36767-3906-4686-A6B3-0F16DECA438D}"/>
   <bookViews>
-    <workbookView xWindow="18450" yWindow="3045" windowWidth="28950" windowHeight="17595" xr2:uid="{0D0EC0D8-2E8F-4565-9EDB-23E86D13F010}"/>
+    <workbookView xWindow="255" yWindow="975" windowWidth="28950" windowHeight="17595" xr2:uid="{0D0EC0D8-2E8F-4565-9EDB-23E86D13F010}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="151">
   <si>
     <t>Category</t>
   </si>
@@ -420,9 +420,6 @@
     <t>Keenovo Silicone AC Heater w/ thermistor - 120x120mm (200W)</t>
   </si>
   <si>
-    <t>Use leadscrews and coupler</t>
-  </si>
-  <si>
     <t>2020x160 (A/B connector back)</t>
   </si>
   <si>
@@ -459,10 +456,46 @@
     <t>180x180 Saladfork/Micron</t>
   </si>
   <si>
-    <t>Try 230 or 225 here</t>
-  </si>
-  <si>
-    <t>Use 240 here</t>
+    <t>289x289x4mm</t>
+  </si>
+  <si>
+    <t>302x372x4mm</t>
+  </si>
+  <si>
+    <t>151.5x373x3mm</t>
+  </si>
+  <si>
+    <t>303x373x3mm</t>
+  </si>
+  <si>
+    <t>303x303x3mm</t>
+  </si>
+  <si>
+    <t>deck/bottom</t>
+  </si>
+  <si>
+    <t>top</t>
+  </si>
+  <si>
+    <t>sides</t>
+  </si>
+  <si>
+    <t>rear</t>
+  </si>
+  <si>
+    <t>front doors</t>
+  </si>
+  <si>
+    <t>Use leadscrews and couplers</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Z - 235mm</t>
   </si>
 </sst>
 </file>
@@ -506,9 +539,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -827,7 +861,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91481DB4-E564-4582-A47E-448BEE3A17E9}">
-  <dimension ref="A1:D115"/>
+  <dimension ref="A1:E115"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.85546875" bestFit="1" customWidth="1"/>
@@ -1128,7 +1162,7 @@
         <v>1</v>
       </c>
       <c r="D35" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -1139,7 +1173,7 @@
         <v>2</v>
       </c>
       <c r="D36" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -1150,7 +1184,7 @@
         <v>3</v>
       </c>
       <c r="D37" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -1383,7 +1417,7 @@
         <v>3</v>
       </c>
       <c r="D65" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
@@ -1646,10 +1680,10 @@
         <v>4</v>
       </c>
       <c r="D96" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B97" t="s">
         <v>107</v>
       </c>
@@ -1657,10 +1691,10 @@
         <v>3</v>
       </c>
       <c r="D97" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B98" t="s">
         <v>111</v>
       </c>
@@ -1668,10 +1702,10 @@
         <v>1</v>
       </c>
       <c r="D98" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B99" t="s">
         <v>107</v>
       </c>
@@ -1679,10 +1713,10 @@
         <v>2</v>
       </c>
       <c r="D99" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B100" t="s">
         <v>107</v>
       </c>
@@ -1690,10 +1724,10 @@
         <v>2</v>
       </c>
       <c r="D100" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B101" t="s">
         <v>107</v>
       </c>
@@ -1701,10 +1735,10 @@
         <v>2</v>
       </c>
       <c r="D101" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B102" t="s">
         <v>108</v>
       </c>
@@ -1712,10 +1746,10 @@
         <v>1</v>
       </c>
       <c r="D102" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B103" t="s">
         <v>106</v>
       </c>
@@ -1723,10 +1757,10 @@
         <v>1</v>
       </c>
       <c r="D103" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B104" t="s">
         <v>109</v>
       </c>
@@ -1734,10 +1768,10 @@
         <v>1</v>
       </c>
       <c r="D104" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B105" t="s">
         <v>112</v>
       </c>
@@ -1745,10 +1779,10 @@
         <v>1</v>
       </c>
       <c r="D105" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B106" t="s">
         <v>113</v>
       </c>
@@ -1756,53 +1790,83 @@
         <v>1</v>
       </c>
       <c r="D106" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>114</v>
       </c>
       <c r="B107" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C107" s="1">
+      <c r="C107" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D107" t="s">
+        <v>137</v>
+      </c>
+      <c r="E107" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B108" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="C108" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C108" s="2">
+        <v>1</v>
+      </c>
+      <c r="D108" t="s">
+        <v>138</v>
+      </c>
+      <c r="E108" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B109" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="C109" s="1">
+      <c r="C109" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D109" t="s">
+        <v>139</v>
+      </c>
+      <c r="E109" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B110" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="C110" s="1">
+      <c r="C110" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D110" t="s">
+        <v>140</v>
+      </c>
+      <c r="E110" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B111" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="C111" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C111" s="2">
+        <v>1</v>
+      </c>
+      <c r="D111" t="s">
+        <v>141</v>
+      </c>
+      <c r="E111" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>120</v>
       </c>
@@ -1813,7 +1877,7 @@
         <v>1</v>
       </c>
       <c r="D112" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="113" spans="2:3" x14ac:dyDescent="0.25">

</xml_diff>